<commit_message>
Atualiza CRONOGRAMA - ASSUNTO.xlsx pelo dashboard
</commit_message>
<xml_diff>
--- a/CRONOGRAMA - ASSUNTO.xlsx
+++ b/CRONOGRAMA - ASSUNTO.xlsx
@@ -26,8 +26,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="166" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -150,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -204,7 +204,8 @@
     <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -918,8 +919,8 @@
           <t>Início do plano</t>
         </is>
       </c>
-      <c r="B2" s="21" t="n">
-        <v>46315</v>
+      <c r="B2" s="22" t="n">
+        <v>46321</v>
       </c>
     </row>
     <row r="4"/>

</xml_diff>